<commit_message>
Add 8-phase enterprise security assessment framework with GitHub Actions workflow and Excel reports
</commit_message>
<xml_diff>
--- a/excel/E2E_Report.xlsx
+++ b/excel/E2E_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="171">
   <si>
     <t>Metric</t>
   </si>
@@ -25,7 +25,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>7/8/2026, 9:16:23 pm</t>
+    <t>7/8/2026, 10:13:06 pm</t>
   </si>
   <si>
     <t>Environment</t>
@@ -67,7 +67,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>187 seconds</t>
+    <t>192 seconds</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -94,7 +94,7 @@
     <t>Duration</t>
   </si>
   <si>
-    <t>TC-2809</t>
+    <t>TC-8378</t>
   </si>
   <si>
     <t>Authentication &amp; Session Management Suite</t>
@@ -106,256 +106,253 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>9:13:17 pm</t>
-  </si>
-  <si>
-    <t>9:13:22 pm</t>
+    <t>10:09:56 pm</t>
+  </si>
+  <si>
+    <t>10:10:02 pm</t>
+  </si>
+  <si>
+    <t>6s</t>
+  </si>
+  <si>
+    <t>TC-6430</t>
+  </si>
+  <si>
+    <t>AUTH-002: Validate login with empty password field</t>
+  </si>
+  <si>
+    <t>10:10:06 pm</t>
+  </si>
+  <si>
+    <t>4s</t>
+  </si>
+  <si>
+    <t>TC-3628</t>
+  </si>
+  <si>
+    <t>AUTH-003: Validate login with invalid credentials</t>
+  </si>
+  <si>
+    <t>10:10:10 pm</t>
+  </si>
+  <si>
+    <t>TC-3216</t>
+  </si>
+  <si>
+    <t>AUTH-004: Validate successful Patient authentication flow</t>
+  </si>
+  <si>
+    <t>10:10:15 pm</t>
   </si>
   <si>
     <t>5s</t>
   </si>
   <si>
-    <t>TC-8857</t>
-  </si>
-  <si>
-    <t>AUTH-002: Validate login with empty password field</t>
-  </si>
-  <si>
-    <t>9:13:27 pm</t>
-  </si>
-  <si>
-    <t>4s</t>
-  </si>
-  <si>
-    <t>TC-3871</t>
-  </si>
-  <si>
-    <t>AUTH-003: Validate login with invalid credentials</t>
-  </si>
-  <si>
-    <t>9:13:31 pm</t>
-  </si>
-  <si>
-    <t>TC-1785</t>
-  </si>
-  <si>
-    <t>AUTH-004: Validate successful Patient authentication flow</t>
-  </si>
-  <si>
-    <t>9:13:35 pm</t>
-  </si>
-  <si>
-    <t>TC-5624</t>
+    <t>TC-5860</t>
   </si>
   <si>
     <t>AUTH-005: Validate Patient logout flow</t>
   </si>
   <si>
-    <t>9:13:40 pm</t>
-  </si>
-  <si>
-    <t>TC-1156</t>
+    <t>10:10:21 pm</t>
+  </si>
+  <si>
+    <t>TC-8000</t>
   </si>
   <si>
     <t>AUTH-006: Validate session persistence on page refresh</t>
   </si>
   <si>
-    <t>9:13:48 pm</t>
+    <t>10:10:28 pm</t>
+  </si>
+  <si>
+    <t>8s</t>
+  </si>
+  <si>
+    <t>TC-7806</t>
+  </si>
+  <si>
+    <t>Dynamic Form Validation &amp; Route Discovery Suite</t>
+  </si>
+  <si>
+    <t>FORM-DYN-001: Validate discovered React routes configuration exists</t>
+  </si>
+  <si>
+    <t>10:10:30 pm</t>
+  </si>
+  <si>
+    <t>2s</t>
+  </si>
+  <si>
+    <t>TC-2418</t>
+  </si>
+  <si>
+    <t>FORM-DYN-002: Dynamic email input format validation on Signup form</t>
+  </si>
+  <si>
+    <t>10:10:47 pm</t>
+  </si>
+  <si>
+    <t>17s</t>
+  </si>
+  <si>
+    <t>TC-1491</t>
+  </si>
+  <si>
+    <t>FORM-DYN-003: Dynamic password mismatch validation on Signup form</t>
+  </si>
+  <si>
+    <t>10:10:51 pm</t>
+  </si>
+  <si>
+    <t>TC-2380</t>
+  </si>
+  <si>
+    <t>FORM-DYN-004: Dynamic validation of Patient Symptom Intake form</t>
+  </si>
+  <si>
+    <t>10:10:59 pm</t>
+  </si>
+  <si>
+    <t>TC-6494</t>
+  </si>
+  <si>
+    <t>FORM-DYN-005: Dynamic validation of Doctor Clinical Notes form</t>
+  </si>
+  <si>
+    <t>10:11:07 pm</t>
+  </si>
+  <si>
+    <t>TC-7378</t>
+  </si>
+  <si>
+    <t>FORM-DYN-006: Dynamic validation of Doctor Prescription Builder form</t>
+  </si>
+  <si>
+    <t>10:11:16 pm</t>
+  </si>
+  <si>
+    <t>9s</t>
+  </si>
+  <si>
+    <t>TC-2445</t>
+  </si>
+  <si>
+    <t>FORM-DYN-007: Dynamic validation of Operations Hospital ICU form</t>
+  </si>
+  <si>
+    <t>10:11:27 pm</t>
+  </si>
+  <si>
+    <t>11s</t>
+  </si>
+  <si>
+    <t>TC-3626</t>
+  </si>
+  <si>
+    <t>End-to-End Multi-Role Healthcare Workflow Suite</t>
+  </si>
+  <si>
+    <t>E2E-001: Execute complete End-to-End patient consultation workflow</t>
+  </si>
+  <si>
+    <t>10:12:07 pm</t>
+  </si>
+  <si>
+    <t>39s</t>
+  </si>
+  <si>
+    <t>TC-9388</t>
+  </si>
+  <si>
+    <t>Navigation &amp; Internal Routing Validation Suite</t>
+  </si>
+  <si>
+    <t>NAV-001: Validate navigation through all Patient workspace links</t>
+  </si>
+  <si>
+    <t>10:12:15 pm</t>
+  </si>
+  <si>
+    <t>TC-6502</t>
+  </si>
+  <si>
+    <t>NAV-002: Validate navigation through Doctor workspace tabs</t>
+  </si>
+  <si>
+    <t>10:12:23 pm</t>
+  </si>
+  <si>
+    <t>TC-8049</t>
+  </si>
+  <si>
+    <t>NAV-003: Validate navigation through Operations workspace tabs</t>
+  </si>
+  <si>
+    <t>10:12:30 pm</t>
+  </si>
+  <si>
+    <t>TC-4845</t>
+  </si>
+  <si>
+    <t>NAV-004: Validate browser refresh, back, and forward navigation</t>
+  </si>
+  <si>
+    <t>10:12:39 pm</t>
+  </si>
+  <si>
+    <t>TC-1256</t>
+  </si>
+  <si>
+    <t>UI &amp; Interactive Elements Validation Suite</t>
+  </si>
+  <si>
+    <t>UI-001: Validate Theme Toggle (Dark / Light mode)</t>
+  </si>
+  <si>
+    <t>10:12:42 pm</t>
+  </si>
+  <si>
+    <t>3s</t>
+  </si>
+  <si>
+    <t>TC-1232</t>
+  </si>
+  <si>
+    <t>UI-002: Validate Language Selector Dropdown</t>
+  </si>
+  <si>
+    <t>10:12:44 pm</t>
+  </si>
+  <si>
+    <t>TC-6884</t>
+  </si>
+  <si>
+    <t>UI-003: Validate Forgot Password Modal open and close</t>
+  </si>
+  <si>
+    <t>10:12:53 pm</t>
+  </si>
+  <si>
+    <t>TC-6956</t>
+  </si>
+  <si>
+    <t>UI-004: Validate Doctor Search Bar filtering in Patient Workspace</t>
+  </si>
+  <si>
+    <t>10:12:59 pm</t>
   </si>
   <si>
     <t>7s</t>
   </si>
   <si>
-    <t>TC-8978</t>
-  </si>
-  <si>
-    <t>Dynamic Form Validation &amp; Route Discovery Suite</t>
-  </si>
-  <si>
-    <t>FORM-DYN-001: Validate discovered React routes configuration exists</t>
-  </si>
-  <si>
-    <t>9:13:50 pm</t>
-  </si>
-  <si>
-    <t>2s</t>
-  </si>
-  <si>
-    <t>TC-7147</t>
-  </si>
-  <si>
-    <t>FORM-DYN-002: Dynamic email input format validation on Signup form</t>
-  </si>
-  <si>
-    <t>9:14:06 pm</t>
-  </si>
-  <si>
-    <t>16s</t>
-  </si>
-  <si>
-    <t>TC-1589</t>
-  </si>
-  <si>
-    <t>FORM-DYN-003: Dynamic password mismatch validation on Signup form</t>
-  </si>
-  <si>
-    <t>9:14:10 pm</t>
-  </si>
-  <si>
-    <t>TC-7669</t>
-  </si>
-  <si>
-    <t>FORM-DYN-004: Dynamic validation of Patient Symptom Intake form</t>
-  </si>
-  <si>
-    <t>9:14:18 pm</t>
-  </si>
-  <si>
-    <t>8s</t>
-  </si>
-  <si>
-    <t>TC-7949</t>
-  </si>
-  <si>
-    <t>FORM-DYN-005: Dynamic validation of Doctor Clinical Notes form</t>
-  </si>
-  <si>
-    <t>9:14:26 pm</t>
-  </si>
-  <si>
-    <t>TC-3681</t>
-  </si>
-  <si>
-    <t>FORM-DYN-006: Dynamic validation of Doctor Prescription Builder form</t>
-  </si>
-  <si>
-    <t>9:14:35 pm</t>
-  </si>
-  <si>
-    <t>9s</t>
-  </si>
-  <si>
-    <t>TC-3095</t>
-  </si>
-  <si>
-    <t>FORM-DYN-007: Dynamic validation of Operations Hospital ICU form</t>
-  </si>
-  <si>
-    <t>9:14:46 pm</t>
-  </si>
-  <si>
-    <t>11s</t>
-  </si>
-  <si>
-    <t>TC-5947</t>
-  </si>
-  <si>
-    <t>End-to-End Multi-Role Healthcare Workflow Suite</t>
-  </si>
-  <si>
-    <t>E2E-001: Execute complete End-to-End patient consultation workflow</t>
-  </si>
-  <si>
-    <t>9:15:24 pm</t>
-  </si>
-  <si>
-    <t>38s</t>
-  </si>
-  <si>
-    <t>TC-1356</t>
-  </si>
-  <si>
-    <t>Navigation &amp; Internal Routing Validation Suite</t>
-  </si>
-  <si>
-    <t>NAV-001: Validate navigation through all Patient workspace links</t>
-  </si>
-  <si>
-    <t>9:15:33 pm</t>
-  </si>
-  <si>
-    <t>TC-5919</t>
-  </si>
-  <si>
-    <t>NAV-002: Validate navigation through Doctor workspace tabs</t>
-  </si>
-  <si>
-    <t>9:15:40 pm</t>
-  </si>
-  <si>
-    <t>TC-6737</t>
-  </si>
-  <si>
-    <t>NAV-003: Validate navigation through Operations workspace tabs</t>
-  </si>
-  <si>
-    <t>9:15:48 pm</t>
-  </si>
-  <si>
-    <t>TC-7552</t>
-  </si>
-  <si>
-    <t>NAV-004: Validate browser refresh, back, and forward navigation</t>
-  </si>
-  <si>
-    <t>9:15:57 pm</t>
-  </si>
-  <si>
-    <t>10s</t>
-  </si>
-  <si>
-    <t>TC-3316</t>
-  </si>
-  <si>
-    <t>UI &amp; Interactive Elements Validation Suite</t>
-  </si>
-  <si>
-    <t>UI-001: Validate Theme Toggle (Dark / Light mode)</t>
-  </si>
-  <si>
-    <t>9:16:00 pm</t>
-  </si>
-  <si>
-    <t>3s</t>
-  </si>
-  <si>
-    <t>TC-7964</t>
-  </si>
-  <si>
-    <t>UI-002: Validate Language Selector Dropdown</t>
-  </si>
-  <si>
-    <t>9:16:02 pm</t>
-  </si>
-  <si>
-    <t>TC-4349</t>
-  </si>
-  <si>
-    <t>UI-003: Validate Forgot Password Modal open and close</t>
-  </si>
-  <si>
-    <t>9:16:10 pm</t>
-  </si>
-  <si>
-    <t>TC-4547</t>
-  </si>
-  <si>
-    <t>UI-004: Validate Doctor Search Bar filtering in Patient Workspace</t>
-  </si>
-  <si>
-    <t>9:16:17 pm</t>
-  </si>
-  <si>
-    <t>TC-6480</t>
+    <t>TC-6371</t>
   </si>
   <si>
     <t>UI-005: Validate Operations Doctor Verification Data Table and Review Modal</t>
   </si>
   <si>
-    <t>9:16:23 pm</t>
-  </si>
-  <si>
-    <t>6s</t>
+    <t>10:13:05 pm</t>
   </si>
   <si>
     <t>Test Name</t>
@@ -388,7 +385,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-08-07 15:43:22</t>
+    <t>2026-08-07 16:40:02</t>
   </si>
   <si>
     <t>Authentication &amp; Session Management Suite AUTH-001: Validate login with empty email field</t>
@@ -400,133 +397,133 @@
     <t>Completed successfully</t>
   </si>
   <si>
-    <t>2026-08-07 15:43:27</t>
+    <t>2026-08-07 16:40:06</t>
   </si>
   <si>
     <t>Authentication &amp; Session Management Suite AUTH-002: Validate login with empty password field</t>
   </si>
   <si>
-    <t>2026-08-07 15:43:31</t>
+    <t>2026-08-07 16:40:10</t>
   </si>
   <si>
     <t>Authentication &amp; Session Management Suite AUTH-003: Validate login with invalid credentials</t>
   </si>
   <si>
-    <t>2026-08-07 15:43:35</t>
+    <t>2026-08-07 16:40:15</t>
   </si>
   <si>
     <t>Authentication &amp; Session Management Suite AUTH-004: Validate successful Patient authentication flow</t>
   </si>
   <si>
-    <t>2026-08-07 15:43:40</t>
+    <t>2026-08-07 16:40:21</t>
   </si>
   <si>
     <t>Authentication &amp; Session Management Suite AUTH-005: Validate Patient logout flow</t>
   </si>
   <si>
-    <t>2026-08-07 15:43:48</t>
+    <t>2026-08-07 16:40:28</t>
   </si>
   <si>
     <t>Authentication &amp; Session Management Suite AUTH-006: Validate session persistence on page refresh</t>
   </si>
   <si>
-    <t>2026-08-07 15:43:50</t>
+    <t>2026-08-07 16:40:30</t>
   </si>
   <si>
     <t>Dynamic Form Validation &amp; Route Discovery Suite FORM-DYN-001: Validate discovered React routes configuration exists</t>
   </si>
   <si>
-    <t>2026-08-07 15:44:06</t>
+    <t>2026-08-07 16:40:47</t>
   </si>
   <si>
     <t>Dynamic Form Validation &amp; Route Discovery Suite FORM-DYN-002: Dynamic email input format validation on Signup form</t>
   </si>
   <si>
-    <t>2026-08-07 15:44:10</t>
+    <t>2026-08-07 16:40:51</t>
   </si>
   <si>
     <t>Dynamic Form Validation &amp; Route Discovery Suite FORM-DYN-003: Dynamic password mismatch validation on Signup form</t>
   </si>
   <si>
-    <t>2026-08-07 15:44:18</t>
+    <t>2026-08-07 16:40:59</t>
   </si>
   <si>
     <t>Dynamic Form Validation &amp; Route Discovery Suite FORM-DYN-004: Dynamic validation of Patient Symptom Intake form</t>
   </si>
   <si>
-    <t>2026-08-07 15:44:26</t>
+    <t>2026-08-07 16:41:07</t>
   </si>
   <si>
     <t>Dynamic Form Validation &amp; Route Discovery Suite FORM-DYN-005: Dynamic validation of Doctor Clinical Notes form</t>
   </si>
   <si>
-    <t>2026-08-07 15:44:35</t>
+    <t>2026-08-07 16:41:16</t>
   </si>
   <si>
     <t>Dynamic Form Validation &amp; Route Discovery Suite FORM-DYN-006: Dynamic validation of Doctor Prescription Builder form</t>
   </si>
   <si>
-    <t>2026-08-07 15:44:46</t>
+    <t>2026-08-07 16:41:27</t>
   </si>
   <si>
     <t>Dynamic Form Validation &amp; Route Discovery Suite FORM-DYN-007: Dynamic validation of Operations Hospital ICU form</t>
   </si>
   <si>
-    <t>2026-08-07 15:45:24</t>
+    <t>2026-08-07 16:42:07</t>
   </si>
   <si>
     <t>End-to-End Multi-Role Healthcare Workflow Suite E2E-001: Execute complete End-to-End patient consultation workflow</t>
   </si>
   <si>
-    <t>2026-08-07 15:45:33</t>
+    <t>2026-08-07 16:42:15</t>
   </si>
   <si>
     <t>Navigation &amp; Internal Routing Validation Suite NAV-001: Validate navigation through all Patient workspace links</t>
   </si>
   <si>
-    <t>2026-08-07 15:45:40</t>
+    <t>2026-08-07 16:42:23</t>
   </si>
   <si>
     <t>Navigation &amp; Internal Routing Validation Suite NAV-002: Validate navigation through Doctor workspace tabs</t>
   </si>
   <si>
-    <t>2026-08-07 15:45:48</t>
+    <t>2026-08-07 16:42:30</t>
   </si>
   <si>
     <t>Navigation &amp; Internal Routing Validation Suite NAV-003: Validate navigation through Operations workspace tabs</t>
   </si>
   <si>
-    <t>2026-08-07 15:45:57</t>
+    <t>2026-08-07 16:42:39</t>
   </si>
   <si>
     <t>Navigation &amp; Internal Routing Validation Suite NAV-004: Validate browser refresh, back, and forward navigation</t>
   </si>
   <si>
-    <t>2026-08-07 15:46:00</t>
+    <t>2026-08-07 16:42:42</t>
   </si>
   <si>
     <t>UI &amp; Interactive Elements Validation Suite UI-001: Validate Theme Toggle (Dark / Light mode)</t>
   </si>
   <si>
-    <t>2026-08-07 15:46:02</t>
+    <t>2026-08-07 16:42:44</t>
   </si>
   <si>
     <t>UI &amp; Interactive Elements Validation Suite UI-002: Validate Language Selector Dropdown</t>
   </si>
   <si>
-    <t>2026-08-07 15:46:10</t>
+    <t>2026-08-07 16:42:53</t>
   </si>
   <si>
     <t>UI &amp; Interactive Elements Validation Suite UI-003: Validate Forgot Password Modal open and close</t>
   </si>
   <si>
-    <t>2026-08-07 15:46:17</t>
+    <t>2026-08-07 16:42:59</t>
   </si>
   <si>
     <t>UI &amp; Interactive Elements Validation Suite UI-004: Validate Doctor Search Bar filtering in Patient Workspace</t>
   </si>
   <si>
-    <t>2026-08-07 15:46:23</t>
+    <t>2026-08-07 16:43:05</t>
   </si>
   <si>
     <t>UI &amp; Interactive Elements Validation Suite UI-005: Validate Operations Doctor Verification Data Table and Review Modal</t>
@@ -1170,18 +1167,18 @@
         <v>42</v>
       </c>
       <c r="H5" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
         <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
@@ -1193,7 +1190,7 @@
         <v>42</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H6" t="s">
         <v>32</v>
@@ -1201,13 +1198,13 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
         <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D7" t="s">
         <v>7</v>
@@ -1216,24 +1213,24 @@
         <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
@@ -1242,24 +1239,24 @@
         <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D9" t="s">
         <v>7</v>
@@ -1268,24 +1265,24 @@
         <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
         <v>7</v>
@@ -1294,10 +1291,10 @@
         <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H10" t="s">
         <v>36</v>
@@ -1305,28 +1302,28 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" t="s">
         <v>62</v>
       </c>
-      <c r="B11" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11" t="s">
-        <v>63</v>
-      </c>
-      <c r="D11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" t="s">
-        <v>61</v>
-      </c>
       <c r="G11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H11" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1334,7 +1331,7 @@
         <v>66</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s">
         <v>67</v>
@@ -1346,13 +1343,13 @@
         <v>29</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G12" t="s">
         <v>68</v>
       </c>
       <c r="H12" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1360,7 +1357,7 @@
         <v>69</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C13" t="s">
         <v>70</v>
@@ -1386,7 +1383,7 @@
         <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
         <v>74</v>
@@ -1456,7 +1453,7 @@
         <v>85</v>
       </c>
       <c r="H16" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1482,7 +1479,7 @@
         <v>88</v>
       </c>
       <c r="H17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1508,7 +1505,7 @@
         <v>91</v>
       </c>
       <c r="H18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1534,18 +1531,18 @@
         <v>94</v>
       </c>
       <c r="H19" t="s">
-        <v>95</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>95</v>
+      </c>
+      <c r="B20" t="s">
         <v>96</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>97</v>
-      </c>
-      <c r="C20" t="s">
-        <v>98</v>
       </c>
       <c r="D20" t="s">
         <v>7</v>
@@ -1557,88 +1554,88 @@
         <v>94</v>
       </c>
       <c r="G20" t="s">
+        <v>98</v>
+      </c>
+      <c r="H20" t="s">
         <v>99</v>
-      </c>
-      <c r="H20" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" t="s">
         <v>101</v>
       </c>
-      <c r="B21" t="s">
-        <v>97</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F21" t="s">
+        <v>98</v>
+      </c>
+      <c r="G21" t="s">
         <v>102</v>
       </c>
-      <c r="D21" t="s">
-        <v>7</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F21" t="s">
-        <v>99</v>
-      </c>
-      <c r="G21" t="s">
-        <v>103</v>
-      </c>
       <c r="H21" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" t="s">
+        <v>96</v>
+      </c>
+      <c r="C22" t="s">
         <v>104</v>
       </c>
-      <c r="B22" t="s">
-        <v>97</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F22" t="s">
+        <v>102</v>
+      </c>
+      <c r="G22" t="s">
         <v>105</v>
       </c>
-      <c r="D22" t="s">
-        <v>7</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F22" t="s">
-        <v>103</v>
-      </c>
-      <c r="G22" t="s">
-        <v>106</v>
-      </c>
       <c r="H22" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>106</v>
+      </c>
+      <c r="B23" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" t="s">
         <v>107</v>
       </c>
-      <c r="B23" t="s">
-        <v>97</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
+        <v>7</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F23" t="s">
+        <v>105</v>
+      </c>
+      <c r="G23" t="s">
         <v>108</v>
       </c>
-      <c r="D23" t="s">
-        <v>7</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F23" t="s">
-        <v>106</v>
-      </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>109</v>
-      </c>
-      <c r="H23" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1646,7 +1643,7 @@
         <v>110</v>
       </c>
       <c r="B24" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C24" t="s">
         <v>111</v>
@@ -1658,13 +1655,13 @@
         <v>29</v>
       </c>
       <c r="F24" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G24" t="s">
         <v>112</v>
       </c>
       <c r="H24" t="s">
-        <v>113</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1687,30 +1684,30 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" t="s">
         <v>118</v>
       </c>
-      <c r="B2" t="s">
-        <v>119</v>
-      </c>
       <c r="C2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -1739,410 +1736,410 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
         <v>124</v>
       </c>
-      <c r="B2" t="s">
-        <v>125</v>
-      </c>
       <c r="C2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D2" t="s">
         <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" t="s">
         <v>128</v>
       </c>
-      <c r="B3" t="s">
-        <v>129</v>
-      </c>
       <c r="C3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D3" t="s">
         <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B4" t="s">
         <v>130</v>
       </c>
-      <c r="B4" t="s">
-        <v>131</v>
-      </c>
       <c r="C4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" t="s">
         <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" t="s">
         <v>132</v>
       </c>
-      <c r="B5" t="s">
-        <v>133</v>
-      </c>
       <c r="C5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D5" t="s">
         <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B6" t="s">
         <v>134</v>
       </c>
-      <c r="B6" t="s">
-        <v>135</v>
-      </c>
       <c r="C6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D6" t="s">
         <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B7" t="s">
         <v>136</v>
       </c>
-      <c r="B7" t="s">
-        <v>137</v>
-      </c>
       <c r="C7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D7" t="s">
         <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" t="s">
         <v>138</v>
       </c>
-      <c r="B8" t="s">
-        <v>139</v>
-      </c>
       <c r="C8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D8" t="s">
         <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B9" t="s">
         <v>140</v>
       </c>
-      <c r="B9" t="s">
-        <v>141</v>
-      </c>
       <c r="C9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D9" t="s">
         <v>29</v>
       </c>
       <c r="E9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B10" t="s">
         <v>142</v>
       </c>
-      <c r="B10" t="s">
-        <v>143</v>
-      </c>
       <c r="C10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D10" t="s">
         <v>29</v>
       </c>
       <c r="E10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B11" t="s">
         <v>144</v>
       </c>
-      <c r="B11" t="s">
-        <v>145</v>
-      </c>
       <c r="C11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D11" t="s">
         <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>145</v>
+      </c>
+      <c r="B12" t="s">
         <v>146</v>
       </c>
-      <c r="B12" t="s">
-        <v>147</v>
-      </c>
       <c r="C12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D12" t="s">
         <v>29</v>
       </c>
       <c r="E12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>147</v>
+      </c>
+      <c r="B13" t="s">
         <v>148</v>
       </c>
-      <c r="B13" t="s">
-        <v>149</v>
-      </c>
       <c r="C13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D13" t="s">
         <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>149</v>
+      </c>
+      <c r="B14" t="s">
         <v>150</v>
       </c>
-      <c r="B14" t="s">
-        <v>151</v>
-      </c>
       <c r="C14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D14" t="s">
         <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>151</v>
+      </c>
+      <c r="B15" t="s">
         <v>152</v>
       </c>
-      <c r="B15" t="s">
-        <v>153</v>
-      </c>
       <c r="C15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D15" t="s">
         <v>29</v>
       </c>
       <c r="E15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>153</v>
+      </c>
+      <c r="B16" t="s">
         <v>154</v>
       </c>
-      <c r="B16" t="s">
-        <v>155</v>
-      </c>
       <c r="C16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D16" t="s">
         <v>29</v>
       </c>
       <c r="E16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>155</v>
+      </c>
+      <c r="B17" t="s">
         <v>156</v>
       </c>
-      <c r="B17" t="s">
-        <v>157</v>
-      </c>
       <c r="C17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D17" t="s">
         <v>29</v>
       </c>
       <c r="E17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>157</v>
+      </c>
+      <c r="B18" t="s">
         <v>158</v>
       </c>
-      <c r="B18" t="s">
-        <v>159</v>
-      </c>
       <c r="C18" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D18" t="s">
         <v>29</v>
       </c>
       <c r="E18" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>159</v>
+      </c>
+      <c r="B19" t="s">
         <v>160</v>
       </c>
-      <c r="B19" t="s">
-        <v>161</v>
-      </c>
       <c r="C19" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D19" t="s">
         <v>29</v>
       </c>
       <c r="E19" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>161</v>
+      </c>
+      <c r="B20" t="s">
         <v>162</v>
       </c>
-      <c r="B20" t="s">
-        <v>163</v>
-      </c>
       <c r="C20" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D20" t="s">
         <v>29</v>
       </c>
       <c r="E20" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>163</v>
+      </c>
+      <c r="B21" t="s">
         <v>164</v>
       </c>
-      <c r="B21" t="s">
-        <v>165</v>
-      </c>
       <c r="C21" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D21" t="s">
         <v>29</v>
       </c>
       <c r="E21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>165</v>
+      </c>
+      <c r="B22" t="s">
         <v>166</v>
       </c>
-      <c r="B22" t="s">
-        <v>167</v>
-      </c>
       <c r="C22" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D22" t="s">
         <v>29</v>
       </c>
       <c r="E22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>167</v>
+      </c>
+      <c r="B23" t="s">
         <v>168</v>
       </c>
-      <c r="B23" t="s">
-        <v>169</v>
-      </c>
       <c r="C23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D23" t="s">
         <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>169</v>
+      </c>
+      <c r="B24" t="s">
         <v>170</v>
       </c>
-      <c r="B24" t="s">
-        <v>171</v>
-      </c>
       <c r="C24" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D24" t="s">
         <v>29</v>
       </c>
       <c r="E24" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>